<commit_message>
fix: Support event participation for non-members (#343)
</commit_message>
<xml_diff>
--- a/__fixtures__/db-screenshot.xlsx
+++ b/__fixtures__/db-screenshot.xlsx
@@ -786,7 +786,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:H15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -796,13 +796,22 @@
         <v>propertyId</v>
       </c>
       <c r="C1" t="str">
+        <v>setIndex</v>
+      </c>
+      <c r="D1" t="str">
         <v>firstName</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>lastName</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>optOut</v>
+      </c>
+      <c r="G1" t="str">
+        <v>moveInDate</v>
+      </c>
+      <c r="H1" t="str">
+        <v>moveOutDate</v>
       </c>
     </row>
     <row r="2">
@@ -812,14 +821,23 @@
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" t="str">
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="str">
         <v>Gaetano</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Hayes</v>
       </c>
-      <c r="E2">
-        <v>1</v>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -829,14 +847,23 @@
       <c r="B3">
         <v>4</v>
       </c>
-      <c r="C3" t="str">
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3" t="str">
         <v>Lonzo</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Hegmann</v>
       </c>
-      <c r="E3">
-        <v>1</v>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -846,14 +873,23 @@
       <c r="B4">
         <v>4</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="str">
         <v>Florian</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Flatley</v>
       </c>
-      <c r="E4">
-        <v>1</v>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -863,14 +899,23 @@
       <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" t="str">
         <v>Conor</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>Stroman</v>
       </c>
-      <c r="E5">
-        <v>1</v>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -880,14 +925,23 @@
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="str">
         <v>Jermey</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>Hegmann</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>0</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -897,14 +951,23 @@
       <c r="B7">
         <v>5</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="str">
         <v>Mia</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>Kiehn</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>0</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -914,14 +977,23 @@
       <c r="B8">
         <v>5</v>
       </c>
-      <c r="C8" t="str">
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8" t="str">
         <v>Stanley</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>Auer</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>0</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -931,14 +1003,23 @@
       <c r="B9">
         <v>6</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9" t="str">
         <v>Kamren</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>Morissette</v>
       </c>
-      <c r="E9">
-        <v>1</v>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -948,14 +1029,23 @@
       <c r="B10">
         <v>6</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10" t="str">
         <v>Rickie</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>Rogahn</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>0</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -965,14 +1055,23 @@
       <c r="B11">
         <v>6</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11" t="str">
         <v>Harvey</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>McLaughlin</v>
       </c>
-      <c r="E11">
-        <v>1</v>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -982,14 +1081,23 @@
       <c r="B12">
         <v>6</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12" t="str">
         <v>Lempi</v>
       </c>
-      <c r="D12" t="str">
+      <c r="E12" t="str">
         <v>Daugherty</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>0</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -999,14 +1107,23 @@
       <c r="B13">
         <v>8</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13" t="str">
         <v>Aubrey</v>
       </c>
-      <c r="D13" t="str">
+      <c r="E13" t="str">
         <v>Stiedemann</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <v>0</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1016,14 +1133,23 @@
       <c r="B14">
         <v>8</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14" t="str">
         <v>Justina</v>
       </c>
-      <c r="D14" t="str">
+      <c r="E14" t="str">
         <v>Reilly</v>
       </c>
-      <c r="E14">
-        <v>1</v>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -1033,19 +1159,28 @@
       <c r="B15">
         <v>8</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15" t="str">
         <v>Savanah</v>
       </c>
-      <c r="D15" t="str">
+      <c r="E15" t="str">
         <v>Kautzer</v>
       </c>
-      <c r="E15">
-        <v>1</v>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2032,7 +2167,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:I41"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2048,12 +2183,18 @@
         <v>isMember</v>
       </c>
       <c r="E1" t="str">
+        <v>price</v>
+      </c>
+      <c r="F1" t="str">
+        <v>paymentEventName</v>
+      </c>
+      <c r="G1" t="str">
+        <v>paymentDate</v>
+      </c>
+      <c r="H1" t="str">
         <v>paymentMethod</v>
       </c>
-      <c r="F1" t="str">
-        <v>price</v>
-      </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>paymentDeposited</v>
       </c>
     </row>
@@ -2085,12 +2226,18 @@
         <v>1</v>
       </c>
       <c r="E3" t="str">
+        <v>20</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Clean-Up</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2024-01-02T00:00:00.000Z</v>
+      </c>
+      <c r="H3" t="str">
         <v>cash</v>
       </c>
-      <c r="F3" t="str">
-        <v>20</v>
-      </c>
-      <c r="G3">
+      <c r="I3">
         <v>1</v>
       </c>
     </row>
@@ -2108,12 +2255,18 @@
         <v>1</v>
       </c>
       <c r="E4" t="str">
+        <v>13</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Community Forum</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2023-10-20T00:00:00.000Z</v>
+      </c>
+      <c r="H4" t="str">
         <v>cash</v>
       </c>
-      <c r="F4" t="str">
-        <v>13</v>
-      </c>
-      <c r="G4">
+      <c r="I4">
         <v>0</v>
       </c>
     </row>
@@ -2215,12 +2368,18 @@
         <v>1</v>
       </c>
       <c r="E11" t="str">
+        <v>19</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Meet &amp; Greet</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2024-05-19T00:00:00.000Z</v>
+      </c>
+      <c r="H11" t="str">
         <v>cash</v>
       </c>
-      <c r="F11" t="str">
-        <v>19</v>
-      </c>
-      <c r="G11">
+      <c r="I11">
         <v>1</v>
       </c>
     </row>
@@ -2252,12 +2411,18 @@
         <v>1</v>
       </c>
       <c r="E13" t="str">
+        <v>13</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Town Hall</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2022-08-01T00:00:00.000Z</v>
+      </c>
+      <c r="H13" t="str">
         <v>e-transfer</v>
       </c>
-      <c r="F13" t="str">
-        <v>13</v>
-      </c>
-      <c r="G13">
+      <c r="I13">
         <v>1</v>
       </c>
     </row>
@@ -2275,12 +2440,18 @@
         <v>1</v>
       </c>
       <c r="E14" t="str">
+        <v>12</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Meet &amp; Greet</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2025-05-03T00:00:00.000Z</v>
+      </c>
+      <c r="H14" t="str">
         <v>cash</v>
       </c>
-      <c r="F14" t="str">
-        <v>12</v>
-      </c>
-      <c r="G14">
+      <c r="I14">
         <v>1</v>
       </c>
     </row>
@@ -2312,12 +2483,18 @@
         <v>1</v>
       </c>
       <c r="E16" t="str">
+        <v>15</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Town Planning Night</v>
+      </c>
+      <c r="G16" t="str">
+        <v>2023-03-15T00:00:00.000Z</v>
+      </c>
+      <c r="H16" t="str">
         <v>e-transfer</v>
       </c>
-      <c r="F16" t="str">
-        <v>15</v>
-      </c>
-      <c r="G16">
+      <c r="I16">
         <v>1</v>
       </c>
     </row>
@@ -2349,12 +2526,18 @@
         <v>1</v>
       </c>
       <c r="E18" t="str">
+        <v>10</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Meet &amp; Greet</v>
+      </c>
+      <c r="G18" t="str">
+        <v>2025-09-20T00:00:00.000Z</v>
+      </c>
+      <c r="H18" t="str">
         <v>cash</v>
       </c>
-      <c r="F18" t="str">
-        <v>10</v>
-      </c>
-      <c r="G18">
+      <c r="I18">
         <v>0</v>
       </c>
     </row>
@@ -2372,12 +2555,18 @@
         <v>1</v>
       </c>
       <c r="E19" t="str">
+        <v>13</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Community Forum</v>
+      </c>
+      <c r="G19" t="str">
+        <v>2024-09-15T00:00:00.000Z</v>
+      </c>
+      <c r="H19" t="str">
         <v>cheque</v>
       </c>
-      <c r="F19" t="str">
-        <v>13</v>
-      </c>
-      <c r="G19">
+      <c r="I19">
         <v>1</v>
       </c>
     </row>
@@ -2395,12 +2584,18 @@
         <v>1</v>
       </c>
       <c r="E20" t="str">
+        <v>19</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Town Planning Night</v>
+      </c>
+      <c r="G20" t="str">
+        <v>2023-02-06T00:00:00.000Z</v>
+      </c>
+      <c r="H20" t="str">
         <v>e-transfer</v>
       </c>
-      <c r="F20" t="str">
-        <v>19</v>
-      </c>
-      <c r="G20">
+      <c r="I20">
         <v>1</v>
       </c>
     </row>
@@ -2432,12 +2627,18 @@
         <v>1</v>
       </c>
       <c r="E22" t="str">
+        <v>10</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Town Hall</v>
+      </c>
+      <c r="G22" t="str">
+        <v>2025-03-12T00:00:00.000Z</v>
+      </c>
+      <c r="H22" t="str">
         <v>e-transfer</v>
       </c>
-      <c r="F22" t="str">
-        <v>10</v>
-      </c>
-      <c r="G22">
+      <c r="I22">
         <v>1</v>
       </c>
     </row>
@@ -2455,12 +2656,18 @@
         <v>1</v>
       </c>
       <c r="E23" t="str">
+        <v>10</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Membership Form</v>
+      </c>
+      <c r="G23" t="str">
+        <v>2024-12-30T00:00:00.000Z</v>
+      </c>
+      <c r="H23" t="str">
         <v>cheque</v>
       </c>
-      <c r="F23" t="str">
-        <v>10</v>
-      </c>
-      <c r="G23">
+      <c r="I23">
         <v>0</v>
       </c>
     </row>
@@ -2520,12 +2727,18 @@
         <v>1</v>
       </c>
       <c r="E27" t="str">
+        <v>19</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Town Hall</v>
+      </c>
+      <c r="G27" t="str">
+        <v>2024-01-20T00:00:00.000Z</v>
+      </c>
+      <c r="H27" t="str">
         <v>cash</v>
       </c>
-      <c r="F27" t="str">
-        <v>19</v>
-      </c>
-      <c r="G27">
+      <c r="I27">
         <v>0</v>
       </c>
     </row>
@@ -2557,12 +2770,18 @@
         <v>1</v>
       </c>
       <c r="E29" t="str">
+        <v>11</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Community Forum</v>
+      </c>
+      <c r="G29" t="str">
+        <v>2022-04-17T00:00:00.000Z</v>
+      </c>
+      <c r="H29" t="str">
         <v>e-transfer</v>
       </c>
-      <c r="F29" t="str">
-        <v>11</v>
-      </c>
-      <c r="G29">
+      <c r="I29">
         <v>1</v>
       </c>
     </row>
@@ -2580,12 +2799,18 @@
         <v>1</v>
       </c>
       <c r="E30" t="str">
+        <v>14</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Town Hall</v>
+      </c>
+      <c r="G30" t="str">
+        <v>2025-02-09T00:00:00.000Z</v>
+      </c>
+      <c r="H30" t="str">
         <v>e-transfer</v>
       </c>
-      <c r="F30" t="str">
-        <v>14</v>
-      </c>
-      <c r="G30">
+      <c r="I30">
         <v>1</v>
       </c>
     </row>
@@ -2603,12 +2828,18 @@
         <v>1</v>
       </c>
       <c r="E31" t="str">
+        <v>15</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Membership Form</v>
+      </c>
+      <c r="G31" t="str">
+        <v>2024-12-28T00:00:00.000Z</v>
+      </c>
+      <c r="H31" t="str">
         <v>cheque</v>
       </c>
-      <c r="F31" t="str">
-        <v>15</v>
-      </c>
-      <c r="G31">
+      <c r="I31">
         <v>0</v>
       </c>
     </row>
@@ -2626,12 +2857,18 @@
         <v>1</v>
       </c>
       <c r="E32" t="str">
+        <v>12</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Membership Form</v>
+      </c>
+      <c r="G32" t="str">
+        <v>2023-06-21T00:00:00.000Z</v>
+      </c>
+      <c r="H32" t="str">
         <v>cheque</v>
       </c>
-      <c r="F32" t="str">
-        <v>12</v>
-      </c>
-      <c r="G32">
+      <c r="I32">
         <v>1</v>
       </c>
     </row>
@@ -2649,12 +2886,18 @@
         <v>1</v>
       </c>
       <c r="E33" t="str">
+        <v>20</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Community Forum</v>
+      </c>
+      <c r="G33" t="str">
+        <v>2022-02-26T00:00:00.000Z</v>
+      </c>
+      <c r="H33" t="str">
         <v>e-transfer</v>
       </c>
-      <c r="F33" t="str">
-        <v>20</v>
-      </c>
-      <c r="G33">
+      <c r="I33">
         <v>1</v>
       </c>
     </row>
@@ -2686,12 +2929,18 @@
         <v>1</v>
       </c>
       <c r="E35" t="str">
+        <v>16</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Town Hall</v>
+      </c>
+      <c r="G35" t="str">
+        <v>2024-09-15T00:00:00.000Z</v>
+      </c>
+      <c r="H35" t="str">
         <v>cash</v>
       </c>
-      <c r="F35" t="str">
-        <v>16</v>
-      </c>
-      <c r="G35">
+      <c r="I35">
         <v>0</v>
       </c>
     </row>
@@ -2723,12 +2972,18 @@
         <v>1</v>
       </c>
       <c r="E37" t="str">
+        <v>12</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Town Planning Night</v>
+      </c>
+      <c r="G37" t="str">
+        <v>2022-08-09T00:00:00.000Z</v>
+      </c>
+      <c r="H37" t="str">
         <v>cash</v>
       </c>
-      <c r="F37" t="str">
-        <v>12</v>
-      </c>
-      <c r="G37">
+      <c r="I37">
         <v>0</v>
       </c>
     </row>
@@ -2746,12 +3001,18 @@
         <v>1</v>
       </c>
       <c r="E38" t="str">
+        <v>14</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Membership Form</v>
+      </c>
+      <c r="G38" t="str">
+        <v>2025-10-04T00:00:00.000Z</v>
+      </c>
+      <c r="H38" t="str">
         <v>cheque</v>
       </c>
-      <c r="F38" t="str">
-        <v>14</v>
-      </c>
-      <c r="G38">
+      <c r="I38">
         <v>0</v>
       </c>
     </row>
@@ -2797,18 +3058,24 @@
         <v>1</v>
       </c>
       <c r="E41" t="str">
+        <v>16</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Town Planning Night</v>
+      </c>
+      <c r="G41" t="str">
+        <v>2022-01-20T00:00:00.000Z</v>
+      </c>
+      <c r="H41" t="str">
         <v>e-transfer</v>
       </c>
-      <c r="F41" t="str">
-        <v>16</v>
-      </c>
-      <c r="G41">
+      <c r="I41">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I41"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3638,7 +3905,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:G87"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3659,6 +3926,9 @@
       <c r="F1" t="str">
         <v>paymentMethod</v>
       </c>
+      <c r="G1" t="str">
+        <v>paymentDate</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -3678,6 +3948,9 @@
       </c>
       <c r="F2" t="str">
         <v>e-transfer</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -3699,6 +3972,9 @@
       <c r="F3" t="str">
         <v>cash</v>
       </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -3719,6 +3995,9 @@
       <c r="F4" t="str">
         <v>cheque</v>
       </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -3739,6 +4018,9 @@
       <c r="F5" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -3759,6 +4041,9 @@
       <c r="F6" t="str">
         <v>cheque</v>
       </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -3779,6 +4064,9 @@
       <c r="F7" t="str">
         <v>cash</v>
       </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -3799,6 +4087,9 @@
       <c r="F8" t="str">
         <v>cheque</v>
       </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -3819,6 +4110,9 @@
       <c r="F9" t="str">
         <v>cash</v>
       </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -3839,6 +4133,9 @@
       <c r="F10" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -3859,6 +4156,9 @@
       <c r="F11" t="str">
         <v>cash</v>
       </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -3879,6 +4179,9 @@
       <c r="F12" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -3899,6 +4202,9 @@
       <c r="F13" t="str">
         <v>cash</v>
       </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -3919,6 +4225,9 @@
       <c r="F14" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -3939,6 +4248,9 @@
       <c r="F15" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -3959,6 +4271,9 @@
       <c r="F16" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -3979,6 +4294,9 @@
       <c r="F17" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -3999,6 +4317,9 @@
       <c r="F18" t="str">
         <v>cash</v>
       </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -4019,6 +4340,9 @@
       <c r="F19" t="str">
         <v>cash</v>
       </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -4039,6 +4363,9 @@
       <c r="F20" t="str">
         <v>cash</v>
       </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -4059,6 +4386,9 @@
       <c r="F21" t="str">
         <v>cash</v>
       </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -4079,6 +4409,9 @@
       <c r="F22" t="str">
         <v>cash</v>
       </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -4099,6 +4432,9 @@
       <c r="F23" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -4119,6 +4455,9 @@
       <c r="F24" t="str">
         <v>cash</v>
       </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -4139,6 +4478,9 @@
       <c r="F25" t="str">
         <v>cash</v>
       </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -4159,6 +4501,9 @@
       <c r="F26" t="str">
         <v>cheque</v>
       </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -4179,6 +4524,9 @@
       <c r="F27" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -4199,6 +4547,9 @@
       <c r="F28" t="str">
         <v>cheque</v>
       </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -4219,6 +4570,9 @@
       <c r="F29" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -4239,6 +4593,9 @@
       <c r="F30" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -4259,6 +4616,9 @@
       <c r="F31" t="str">
         <v>cheque</v>
       </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -4279,6 +4639,9 @@
       <c r="F32" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -4299,6 +4662,9 @@
       <c r="F33" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -4319,6 +4685,9 @@
       <c r="F34" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -4339,6 +4708,9 @@
       <c r="F35" t="str">
         <v>cheque</v>
       </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -4359,6 +4731,9 @@
       <c r="F36" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -4379,6 +4754,9 @@
       <c r="F37" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -4399,6 +4777,9 @@
       <c r="F38" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -4419,6 +4800,9 @@
       <c r="F39" t="str">
         <v>cheque</v>
       </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -4439,6 +4823,9 @@
       <c r="F40" t="str">
         <v>cash</v>
       </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -4459,6 +4846,9 @@
       <c r="F41" t="str">
         <v>cash</v>
       </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -4479,6 +4869,9 @@
       <c r="F42" t="str">
         <v>cash</v>
       </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -4499,6 +4892,9 @@
       <c r="F43" t="str">
         <v>cash</v>
       </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -4519,6 +4915,9 @@
       <c r="F44" t="str">
         <v>cheque</v>
       </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -4539,6 +4938,9 @@
       <c r="F45" t="str">
         <v>cheque</v>
       </c>
+      <c r="G45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -4559,6 +4961,9 @@
       <c r="F46" t="str">
         <v>cheque</v>
       </c>
+      <c r="G46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -4579,6 +4984,9 @@
       <c r="F47" t="str">
         <v>cheque</v>
       </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -4599,6 +5007,9 @@
       <c r="F48" t="str">
         <v>cash</v>
       </c>
+      <c r="G48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -4619,6 +5030,9 @@
       <c r="F49" t="str">
         <v>cash</v>
       </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -4639,6 +5053,9 @@
       <c r="F50" t="str">
         <v>cheque</v>
       </c>
+      <c r="G50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -4659,6 +5076,9 @@
       <c r="F51" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -4679,6 +5099,9 @@
       <c r="F52" t="str">
         <v>cash</v>
       </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -4699,6 +5122,9 @@
       <c r="F53" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -4719,6 +5145,9 @@
       <c r="F54" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -4739,6 +5168,9 @@
       <c r="F55" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -4759,6 +5191,9 @@
       <c r="F56" t="str">
         <v>cash</v>
       </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -4779,6 +5214,9 @@
       <c r="F57" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -4799,6 +5237,9 @@
       <c r="F58" t="str">
         <v>cash</v>
       </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -4819,6 +5260,9 @@
       <c r="F59" t="str">
         <v>cash</v>
       </c>
+      <c r="G59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -4839,6 +5283,9 @@
       <c r="F60" t="str">
         <v>cheque</v>
       </c>
+      <c r="G60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -4859,6 +5306,9 @@
       <c r="F61" t="str">
         <v>cheque</v>
       </c>
+      <c r="G61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62">
@@ -4879,6 +5329,9 @@
       <c r="F62" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -4899,6 +5352,9 @@
       <c r="F63" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -4919,6 +5375,9 @@
       <c r="F64" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65">
@@ -4939,6 +5398,9 @@
       <c r="F65" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66">
@@ -4959,6 +5421,9 @@
       <c r="F66" t="str">
         <v>cash</v>
       </c>
+      <c r="G66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67">
@@ -4979,6 +5444,9 @@
       <c r="F67" t="str">
         <v>cash</v>
       </c>
+      <c r="G67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68">
@@ -4999,6 +5467,9 @@
       <c r="F68" t="str">
         <v>cheque</v>
       </c>
+      <c r="G68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69">
@@ -5019,6 +5490,9 @@
       <c r="F69" t="str">
         <v>cash</v>
       </c>
+      <c r="G69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70">
@@ -5039,6 +5513,9 @@
       <c r="F70" t="str">
         <v>cheque</v>
       </c>
+      <c r="G70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71">
@@ -5059,6 +5536,9 @@
       <c r="F71" t="str">
         <v>cheque</v>
       </c>
+      <c r="G71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72">
@@ -5079,6 +5559,9 @@
       <c r="F72" t="str">
         <v>cash</v>
       </c>
+      <c r="G72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73">
@@ -5099,6 +5582,9 @@
       <c r="F73" t="str">
         <v>cheque</v>
       </c>
+      <c r="G73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74">
@@ -5119,6 +5605,9 @@
       <c r="F74" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75">
@@ -5139,6 +5628,9 @@
       <c r="F75" t="str">
         <v>cheque</v>
       </c>
+      <c r="G75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76">
@@ -5159,6 +5651,9 @@
       <c r="F76" t="str">
         <v>cash</v>
       </c>
+      <c r="G76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77">
@@ -5179,6 +5674,9 @@
       <c r="F77" t="str">
         <v>cash</v>
       </c>
+      <c r="G77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78">
@@ -5199,6 +5697,9 @@
       <c r="F78" t="str">
         <v>cash</v>
       </c>
+      <c r="G78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79">
@@ -5219,6 +5720,9 @@
       <c r="F79" t="str">
         <v>cash</v>
       </c>
+      <c r="G79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80">
@@ -5239,6 +5743,9 @@
       <c r="F80" t="str">
         <v>cash</v>
       </c>
+      <c r="G80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81">
@@ -5259,6 +5766,9 @@
       <c r="F81" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82">
@@ -5279,6 +5789,9 @@
       <c r="F82" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83">
@@ -5299,6 +5812,9 @@
       <c r="F83" t="str">
         <v>cash</v>
       </c>
+      <c r="G83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84">
@@ -5319,6 +5835,9 @@
       <c r="F84" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85">
@@ -5339,6 +5858,9 @@
       <c r="F85" t="str">
         <v>cheque</v>
       </c>
+      <c r="G85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86">
@@ -5359,6 +5881,9 @@
       <c r="F86" t="str">
         <v>e-transfer</v>
       </c>
+      <c r="G86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87">
@@ -5379,10 +5904,13 @@
       <c r="F87" t="str">
         <v>cheque</v>
       </c>
+      <c r="G87" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F87"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G87"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>